<commit_message>
paper: finalize native Excel figure layout
</commit_message>
<xml_diff>
--- a/docs/paper/submission_assets/excel/Figure2_E2E_performance.xlsx
+++ b/docs/paper/submission_assets/excel/Figure2_E2E_performance.xlsx
@@ -13,14 +13,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">RawRuns!$A$1:$L$16</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">Figure!$A$1:$J$72</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">Figure!$A$1:$J$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="86">
   <si>
     <t>variant</t>
   </si>
@@ -278,12 +278,6 @@
   </si>
   <si>
     <t>−4.03%</t>
-  </si>
-  <si>
-    <t>图2　三条路径的端到端性能（原生 Excel 图表组合）</t>
-  </si>
-  <si>
-    <t>三个图表均为可编辑的 Excel 原生图表；数值表见 DisplayValues。</t>
   </si>
 </sst>
 </file>
@@ -417,7 +411,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1000" b="1" baseline="0">
+              <a:defRPr sz="900" b="0" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="111827"/>
                 </a:solidFill>
@@ -425,14 +419,13 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1000" b="1" baseline="0">
+              <a:rPr lang="en-US" sz="900" b="0" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="111827"/>
                 </a:solidFill>
                 <a:latin typeface="Microsoft YaHei"/>
               </a:rPr>
-              <a:t>(a) FPS（均值±样本SD；每路径5进程）
-V0→V2R  2.24×；V2R→V3R  +4.07%</a:t>
+              <a:t>V0→V2R  2.24×；V2R→V3R  +4.07%</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -594,7 +587,43 @@
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="111827"/>
+                    </a:solidFill>
+                    <a:latin typeface="Microsoft YaHei"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="900" b="0" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="111827"/>
+                    </a:solidFill>
+                    <a:latin typeface="Microsoft YaHei"/>
+                  </a:rPr>
+                  <a:t>(a) FPS（均值±样本SD；每路径5进程）</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
+        <c:majorTickMark val="in"/>
         <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="12700">
+            <a:solidFill>
+              <a:srgbClr val="111827"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
@@ -652,7 +681,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="in"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -717,7 +746,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1000" b="1" baseline="0">
+              <a:defRPr sz="900" b="0" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="111827"/>
                 </a:solidFill>
@@ -725,14 +754,13 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1000" b="1" baseline="0">
+              <a:rPr lang="en-US" sz="900" b="0" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="111827"/>
                 </a:solidFill>
                 <a:latin typeface="Microsoft YaHei"/>
               </a:rPr>
-              <a:t>(b) 合并样本平均 E2E 延迟（n=5400/路径）
-V0→V2R  −55.45%；V2R→V3R  −4.03%</a:t>
+              <a:t>V0→V2R  −55.45%；V2R→V3R  −4.03%</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -865,7 +893,43 @@
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="111827"/>
+                    </a:solidFill>
+                    <a:latin typeface="Microsoft YaHei"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="900" b="0" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="111827"/>
+                    </a:solidFill>
+                    <a:latin typeface="Microsoft YaHei"/>
+                  </a:rPr>
+                  <a:t>(b) 合并样本平均 E2E 延迟（n=5400/路径）</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
+        <c:majorTickMark val="in"/>
         <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="12700">
+            <a:solidFill>
+              <a:srgbClr val="111827"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
@@ -923,7 +987,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="in"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -981,34 +1045,6 @@
   <c:lang val="en-US"/>
   <c:style val="10"/>
   <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1000" b="1" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="111827"/>
-                </a:solidFill>
-                <a:latin typeface="Microsoft YaHei"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="1000" b="1" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="111827"/>
-                </a:solidFill>
-                <a:latin typeface="Microsoft YaHei"/>
-              </a:rPr>
-              <a:t>(c) 合并样本 P95 / P99（n=5400/路径）</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:layout/>
-    </c:title>
     <c:plotArea>
       <c:layout/>
       <c:barChart>
@@ -1224,7 +1260,43 @@
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="111827"/>
+                    </a:solidFill>
+                    <a:latin typeface="Microsoft YaHei"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="900" b="0" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="111827"/>
+                    </a:solidFill>
+                    <a:latin typeface="Microsoft YaHei"/>
+                  </a:rPr>
+                  <a:t>(c) 合并样本 P95 / P99（n=5400/路径）</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
+        <c:majorTickMark val="in"/>
         <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="12700">
+            <a:solidFill>
+              <a:srgbClr val="111827"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
@@ -1282,7 +1354,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="in"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -1357,14 +1429,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>542925</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1393,8 +1465,8 @@
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>542925</xdr:colOff>
-      <xdr:row>42</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1417,14 +1489,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>47</xdr:row>
+      <xdr:row>50</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>542925</xdr:colOff>
-      <xdr:row>64</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2586,26 +2658,15 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:B2"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="2.7109375" customWidth="1"/>
     <col min="2" max="10" width="12.7109375" customWidth="1"/>
   </cols>
-  <sheetData>
-    <row r="1" spans="2:2">
-      <c r="B1" s="5" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="2" spans="2:2">
-      <c r="B2" s="6" t="s">
-        <v>87</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>
-  <pageSetup fitToHeight="2" orientation="landscape"/>
+  <pageSetup fitToHeight="3" orientation="landscape"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
paper: tighten native Excel figure layout and clear panel captions
</commit_message>
<xml_diff>
--- a/docs/paper/submission_assets/excel/Figure2_E2E_performance.xlsx
+++ b/docs/paper/submission_assets/excel/Figure2_E2E_performance.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">RawRuns!$A$1:$L$16</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">Figure!$A$1:$J$77</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">Figure!$A$1:$J$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,17 @@
       <c:layout/>
     </c:title>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.13"/>
+          <c:y val="0.17999999999999999"/>
+          <c:w val="0.81999999999999995"/>
+          <c:h val="0.56999999999999995"/>
+        </c:manualLayout>
+      </c:layout>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
@@ -768,7 +778,17 @@
       <c:layout/>
     </c:title>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.13"/>
+          <c:y val="0.17999999999999999"/>
+          <c:w val="0.81999999999999995"/>
+          <c:h val="0.56999999999999995"/>
+        </c:manualLayout>
+      </c:layout>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
@@ -1046,7 +1066,17 @@
   <c:style val="10"/>
   <c:chart>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.13"/>
+          <c:y val="0.080000000000000002"/>
+          <c:w val="0.81999999999999995"/>
+          <c:h val="0.56000000000000005"/>
+        </c:manualLayout>
+      </c:layout>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
@@ -1435,7 +1465,7 @@
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>542925</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1459,13 +1489,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>18</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>542925</xdr:colOff>
-      <xdr:row>43</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1489,13 +1519,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>36</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>542925</xdr:colOff>
-      <xdr:row>69</xdr:row>
+      <xdr:row>54</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -2666,7 +2696,7 @@
   </cols>
   <sheetData/>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>
-  <pageSetup fitToHeight="3" orientation="landscape"/>
+  <pageSetup fitToHeight="2" orientation="landscape"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
paper: tighten native Excel chart canvas and separate panel captions
</commit_message>
<xml_diff>
--- a/docs/paper/submission_assets/excel/Figure2_E2E_performance.xlsx
+++ b/docs/paper/submission_assets/excel/Figure2_E2E_performance.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">RawRuns!$A$1:$L$16</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">Figure!$A$1:$J$55</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">Figure!$A$1:$J$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -438,10 +438,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.13"/>
-          <c:y val="0.17999999999999999"/>
-          <c:w val="0.81999999999999995"/>
-          <c:h val="0.56999999999999995"/>
+          <c:x val="0.10000000000000001"/>
+          <c:y val="0.16"/>
+          <c:w val="0.87"/>
+          <c:h val="0.62"/>
         </c:manualLayout>
       </c:layout>
       <c:barChart>
@@ -623,7 +623,14 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.34000000000000002"/>
+              <c:y val="0.88"/>
+            </c:manualLayout>
+          </c:layout>
         </c:title>
         <c:majorTickMark val="in"/>
         <c:tickLblPos val="nextTo"/>
@@ -783,10 +790,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.13"/>
-          <c:y val="0.17999999999999999"/>
-          <c:w val="0.81999999999999995"/>
-          <c:h val="0.56999999999999995"/>
+          <c:x val="0.10000000000000001"/>
+          <c:y val="0.16"/>
+          <c:w val="0.87"/>
+          <c:h val="0.62"/>
         </c:manualLayout>
       </c:layout>
       <c:barChart>
@@ -939,7 +946,14 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.33000000000000002"/>
+              <c:y val="0.88"/>
+            </c:manualLayout>
+          </c:layout>
         </c:title>
         <c:majorTickMark val="in"/>
         <c:tickLblPos val="nextTo"/>
@@ -1071,10 +1085,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.13"/>
-          <c:y val="0.080000000000000002"/>
-          <c:w val="0.81999999999999995"/>
-          <c:h val="0.56000000000000005"/>
+          <c:x val="0.10000000000000001"/>
+          <c:y val="0.059999999999999998"/>
+          <c:w val="0.87"/>
+          <c:h val="0.62"/>
         </c:manualLayout>
       </c:layout>
       <c:barChart>
@@ -1316,7 +1330,14 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.34000000000000002"/>
+              <c:y val="0.75"/>
+            </c:manualLayout>
+          </c:layout>
         </c:title>
         <c:majorTickMark val="in"/>
         <c:tickLblPos val="nextTo"/>
@@ -1465,8 +1486,8 @@
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>542925</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1489,14 +1510,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>542925</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1519,14 +1540,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>36</xdr:row>
+      <xdr:row>34</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>542925</xdr:colOff>
-      <xdr:row>54</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>